<commit_message>
Deploying to gh-pages from @ pedalboard/pedalboard-hw@99058ce3b2bc7db122aa04b2066b6492c6121c5a 🚀
</commit_message>
<xml_diff>
--- a/latest/BoM/Costs/pedalboard-hw-bom.xlsx
+++ b/latest/BoM/Costs/pedalboard-hw-bom.xlsx
@@ -290,7 +290,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1242" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1242" uniqueCount="394">
   <si>
     <t>Row</t>
   </si>
@@ -535,9 +535,6 @@
     <t>LED_0805_2012Metric</t>
   </si>
   <si>
-    <t>~</t>
-  </si>
-  <si>
     <t>https://www.digikey.ch/en/products/detail/harvatek-corporation/B1701URO-20D000114U1930/16671739</t>
   </si>
   <si>
@@ -730,9 +727,6 @@
     <t>https://www.molex.com/en-us/products/part-detail/676433910?display=pdf</t>
   </si>
   <si>
-    <t>https://www.digikey.ch/de/products/detail/molex/0676433910/3598521</t>
-  </si>
-  <si>
     <t>21</t>
   </si>
   <si>
@@ -748,9 +742,6 @@
     <t>https://cdn.amphenol-cs.com/media/wysiwyg/files/drawing/10103594.pdf</t>
   </si>
   <si>
-    <t>https://www.digikey.ch/de/products/detail/amphenol-cs-fci/10103594-0001LF/2350351</t>
-  </si>
-  <si>
     <t>L_Ferrite</t>
   </si>
   <si>
@@ -1264,7 +1255,7 @@
     <t>KiCad Version:</t>
   </si>
   <si>
-    <t>9.0.7+1</t>
+    <t>10.0.1-10.0.1~ubuntu25.10.1</t>
   </si>
   <si>
     <t>Component Groups:</t>
@@ -1429,10 +1420,10 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2026-04-21 20:43:40</t>
-  </si>
-  <si>
-    <t>KiCost® v1.1.20 + KiBot v1.8.5</t>
+    <t>2026-04-22 19:59:05</t>
+  </si>
+  <si>
+    <t>KiCost® v1.1.20 + KiBot v1.8.6</t>
   </si>
   <si>
     <t>5-pin DIN connector (5-pin DIN-5 stereo)</t>
@@ -2333,7 +2324,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="32" customHeight="1">
       <c r="C1" s="1" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -2351,13 +2342,13 @@
     </row>
     <row r="2" spans="1:16">
       <c r="C2" s="2" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="F2" s="3">
         <v>55</v>
@@ -2365,41 +2356,41 @@
     </row>
     <row r="3" spans="1:16">
       <c r="C3" s="2" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="4" spans="1:16">
       <c r="C4" s="2" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="5" spans="1:16">
       <c r="C5" s="2" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="F5" s="3">
         <v>1</v>
@@ -2407,13 +2398,13 @@
     </row>
     <row r="6" spans="1:16">
       <c r="C6" s="2" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="F6" s="3">
         <v>128</v>
@@ -2945,19 +2936,19 @@
         <v>23</v>
       </c>
       <c r="I18" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="J18" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="J18" s="12" t="s">
+      <c r="K18" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L18" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M18" s="12" t="s">
         <v>82</v>
-      </c>
-      <c r="K18" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="L18" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="M18" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="N18" s="10" t="s">
         <v>17</v>
@@ -2971,7 +2962,7 @@
     </row>
     <row r="19" spans="1:16" ht="30" customHeight="1">
       <c r="A19" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>17</v>
@@ -2980,10 +2971,10 @@
         <v>77</v>
       </c>
       <c r="D19" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="E19" s="7" t="s">
         <v>85</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>86</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>80</v>
@@ -2995,10 +2986,10 @@
         <v>23</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="K19" s="6" t="s">
         <v>17</v>
@@ -3007,7 +2998,7 @@
         <v>17</v>
       </c>
       <c r="M19" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="N19" s="6" t="s">
         <v>17</v>
@@ -3021,22 +3012,22 @@
     </row>
     <row r="20" spans="1:16" ht="30" customHeight="1">
       <c r="A20" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="B20" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C20" s="11" t="s">
+      <c r="D20" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="E20" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="F20" s="11" t="s">
         <v>91</v>
-      </c>
-      <c r="F20" s="11" t="s">
-        <v>92</v>
       </c>
       <c r="G20" s="9" t="s">
         <v>16</v>
@@ -3045,10 +3036,10 @@
         <v>23</v>
       </c>
       <c r="I20" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="J20" s="12" t="s">
         <v>93</v>
-      </c>
-      <c r="J20" s="12" t="s">
-        <v>94</v>
       </c>
       <c r="K20" s="10" t="s">
         <v>17</v>
@@ -3071,22 +3062,22 @@
     </row>
     <row r="21" spans="1:16" ht="30" customHeight="1">
       <c r="A21" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C21" s="7" t="s">
+      <c r="D21" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="E21" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="F21" s="7" t="s">
         <v>98</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>99</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>16</v>
@@ -3095,10 +3086,10 @@
         <v>23</v>
       </c>
       <c r="I21" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J21" s="8" t="s">
         <v>100</v>
-      </c>
-      <c r="J21" s="8" t="s">
-        <v>101</v>
       </c>
       <c r="K21" s="6" t="s">
         <v>17</v>
@@ -3121,22 +3112,22 @@
     </row>
     <row r="22" spans="1:16" ht="30" customHeight="1">
       <c r="A22" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="B22" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="11" t="s">
+      <c r="D22" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="E22" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="F22" s="11" t="s">
         <v>105</v>
-      </c>
-      <c r="F22" s="11" t="s">
-        <v>106</v>
       </c>
       <c r="G22" s="9" t="s">
         <v>16</v>
@@ -3145,10 +3136,10 @@
         <v>23</v>
       </c>
       <c r="I22" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="J22" s="12" t="s">
         <v>107</v>
-      </c>
-      <c r="J22" s="12" t="s">
-        <v>108</v>
       </c>
       <c r="K22" s="10" t="s">
         <v>17</v>
@@ -3171,22 +3162,22 @@
     </row>
     <row r="23" spans="1:16" ht="30" customHeight="1">
       <c r="A23" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C23" s="7" t="s">
+      <c r="D23" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="E23" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="F23" s="7" t="s">
         <v>112</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>113</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>16</v>
@@ -3195,10 +3186,10 @@
         <v>23</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="K23" s="6" t="s">
         <v>17</v>
@@ -3221,22 +3212,22 @@
     </row>
     <row r="24" spans="1:16" ht="30" customHeight="1">
       <c r="A24" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="B24" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C24" s="11" t="s">
+      <c r="D24" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="E24" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="E24" s="11" t="s">
+      <c r="F24" s="11" t="s">
         <v>118</v>
-      </c>
-      <c r="F24" s="11" t="s">
-        <v>119</v>
       </c>
       <c r="G24" s="9" t="s">
         <v>22</v>
@@ -3245,13 +3236,13 @@
         <v>23</v>
       </c>
       <c r="I24" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="J24" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="J24" s="12" t="s">
+      <c r="K24" s="12" t="s">
         <v>121</v>
-      </c>
-      <c r="K24" s="12" t="s">
-        <v>122</v>
       </c>
       <c r="L24" s="10" t="s">
         <v>17</v>
@@ -3277,16 +3268,16 @@
         <v>17</v>
       </c>
       <c r="C25" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="E25" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="F25" s="7" t="s">
         <v>125</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>126</v>
       </c>
       <c r="G25" s="5" t="s">
         <v>50</v>
@@ -3295,13 +3286,13 @@
         <v>23</v>
       </c>
       <c r="I25" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="J25" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="J25" s="8" t="s">
+      <c r="K25" s="8" t="s">
         <v>128</v>
-      </c>
-      <c r="K25" s="8" t="s">
-        <v>129</v>
       </c>
       <c r="L25" s="6" t="s">
         <v>17</v>
@@ -3321,22 +3312,22 @@
     </row>
     <row r="26" spans="1:16">
       <c r="A26" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="B26" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C26" s="11" t="s">
+      <c r="D26" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="E26" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="E26" s="11" t="s">
+      <c r="F26" s="11" t="s">
         <v>133</v>
-      </c>
-      <c r="F26" s="11" t="s">
-        <v>134</v>
       </c>
       <c r="G26" s="9" t="s">
         <v>16</v>
@@ -3345,7 +3336,7 @@
         <v>23</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="J26" s="10" t="s">
         <v>17</v>
@@ -3371,22 +3362,22 @@
     </row>
     <row r="27" spans="1:16" ht="30" customHeight="1">
       <c r="A27" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C27" s="7" t="s">
+      <c r="D27" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="E27" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="F27" s="7" t="s">
         <v>137</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>138</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>16</v>
@@ -3395,10 +3386,10 @@
         <v>23</v>
       </c>
       <c r="I27" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="J27" s="8" t="s">
         <v>139</v>
-      </c>
-      <c r="J27" s="8" t="s">
-        <v>140</v>
       </c>
       <c r="K27" s="6" t="s">
         <v>17</v>
@@ -3421,22 +3412,22 @@
     </row>
     <row r="28" spans="1:16" ht="30" customHeight="1">
       <c r="A28" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C28" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="B28" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C28" s="11" t="s">
+      <c r="D28" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="D28" s="11" t="s">
+      <c r="E28" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="F28" s="11" t="s">
         <v>143</v>
-      </c>
-      <c r="E28" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="F28" s="11" t="s">
-        <v>144</v>
       </c>
       <c r="G28" s="9" t="s">
         <v>16</v>
@@ -3445,10 +3436,10 @@
         <v>23</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="J28" s="12" t="s">
-        <v>146</v>
+        <v>144</v>
+      </c>
+      <c r="J28" s="10" t="s">
+        <v>17</v>
       </c>
       <c r="K28" s="10" t="s">
         <v>17</v>
@@ -3471,22 +3462,22 @@
     </row>
     <row r="29" spans="1:16" ht="30" customHeight="1">
       <c r="A29" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="D29" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="B29" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C29" s="7" t="s">
+      <c r="E29" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="F29" s="7" t="s">
         <v>148</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="E29" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>150</v>
       </c>
       <c r="G29" s="5" t="s">
         <v>16</v>
@@ -3495,10 +3486,10 @@
         <v>23</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="J29" s="8" t="s">
-        <v>152</v>
+        <v>149</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>17</v>
       </c>
       <c r="K29" s="6" t="s">
         <v>17</v>
@@ -3527,16 +3518,16 @@
         <v>17</v>
       </c>
       <c r="C30" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D30" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="E30" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="F30" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="D30" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E30" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="F30" s="11" t="s">
-        <v>156</v>
       </c>
       <c r="G30" s="9" t="s">
         <v>33</v>
@@ -3545,10 +3536,10 @@
         <v>23</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="J30" s="12" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="K30" s="10" t="s">
         <v>17</v>
@@ -3571,22 +3562,22 @@
     </row>
     <row r="31" spans="1:16" ht="30" customHeight="1">
       <c r="A31" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="E31" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="B31" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C31" s="7" t="s">
+      <c r="F31" s="7" t="s">
         <v>160</v>
-      </c>
-      <c r="D31" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="E31" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>163</v>
       </c>
       <c r="G31" s="5" t="s">
         <v>16</v>
@@ -3595,13 +3586,13 @@
         <v>23</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="J31" s="8" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="K31" s="8" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="L31" s="6" t="s">
         <v>17</v>
@@ -3621,22 +3612,22 @@
     </row>
     <row r="32" spans="1:16" ht="30" customHeight="1">
       <c r="A32" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="D32" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F32" s="11" t="s">
         <v>167</v>
-      </c>
-      <c r="B32" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C32" s="11" t="s">
-        <v>168</v>
-      </c>
-      <c r="D32" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>168</v>
-      </c>
-      <c r="F32" s="11" t="s">
-        <v>170</v>
       </c>
       <c r="G32" s="9" t="s">
         <v>16</v>
@@ -3645,10 +3636,10 @@
         <v>23</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="J32" s="12" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="K32" s="10" t="s">
         <v>17</v>
@@ -3671,22 +3662,22 @@
     </row>
     <row r="33" spans="1:16" ht="30" customHeight="1">
       <c r="A33" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="E33" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="B33" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C33" s="7" t="s">
+      <c r="F33" s="7" t="s">
         <v>174</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="E33" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="F33" s="7" t="s">
-        <v>177</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>22</v>
@@ -3695,13 +3686,13 @@
         <v>23</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="J33" s="8" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="K33" s="8" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="L33" s="6" t="s">
         <v>17</v>
@@ -3721,22 +3712,22 @@
     </row>
     <row r="34" spans="1:16" ht="30" customHeight="1">
       <c r="A34" s="9" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B34" s="10" t="s">
         <v>17</v>
       </c>
       <c r="C34" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="F34" s="11" t="s">
         <v>174</v>
-      </c>
-      <c r="D34" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="E34" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="F34" s="11" t="s">
-        <v>177</v>
       </c>
       <c r="G34" s="9" t="s">
         <v>22</v>
@@ -3745,10 +3736,10 @@
         <v>23</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="J34" s="12" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="K34" s="10" t="s">
         <v>17</v>
@@ -3771,22 +3762,22 @@
     </row>
     <row r="35" spans="1:16" ht="30" customHeight="1">
       <c r="A35" s="5" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C35" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="F35" s="7" t="s">
         <v>174</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="E35" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="F35" s="7" t="s">
-        <v>177</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>16</v>
@@ -3795,10 +3786,10 @@
         <v>23</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="J35" s="8" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="K35" s="6" t="s">
         <v>17</v>
@@ -3821,22 +3812,22 @@
     </row>
     <row r="36" spans="1:16" ht="30" customHeight="1">
       <c r="A36" s="9" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B36" s="10" t="s">
         <v>17</v>
       </c>
       <c r="C36" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="D36" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="E36" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="F36" s="11" t="s">
         <v>174</v>
-      </c>
-      <c r="D36" s="11" t="s">
-        <v>189</v>
-      </c>
-      <c r="E36" s="11" t="s">
-        <v>190</v>
-      </c>
-      <c r="F36" s="11" t="s">
-        <v>177</v>
       </c>
       <c r="G36" s="9" t="s">
         <v>30</v>
@@ -3845,10 +3836,10 @@
         <v>23</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="J36" s="12" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="K36" s="10" t="s">
         <v>17</v>
@@ -3871,22 +3862,22 @@
     </row>
     <row r="37" spans="1:16" ht="30" customHeight="1">
       <c r="A37" s="5" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C37" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="F37" s="7" t="s">
         <v>174</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="E37" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="F37" s="7" t="s">
-        <v>177</v>
       </c>
       <c r="G37" s="5" t="s">
         <v>42</v>
@@ -3895,10 +3886,10 @@
         <v>23</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="J37" s="8" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="K37" s="6" t="s">
         <v>17</v>
@@ -3921,22 +3912,22 @@
     </row>
     <row r="38" spans="1:16" ht="30" customHeight="1">
       <c r="A38" s="9" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B38" s="10" t="s">
         <v>17</v>
       </c>
       <c r="C38" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="D38" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="E38" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="F38" s="11" t="s">
         <v>174</v>
-      </c>
-      <c r="D38" s="11" t="s">
-        <v>197</v>
-      </c>
-      <c r="E38" s="11" t="s">
-        <v>198</v>
-      </c>
-      <c r="F38" s="11" t="s">
-        <v>177</v>
       </c>
       <c r="G38" s="9" t="s">
         <v>42</v>
@@ -3945,13 +3936,13 @@
         <v>23</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="J38" s="12" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="K38" s="12" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="L38" s="10" t="s">
         <v>17</v>
@@ -3971,22 +3962,22 @@
     </row>
     <row r="39" spans="1:16" ht="30" customHeight="1">
       <c r="A39" s="5" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C39" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="F39" s="7" t="s">
         <v>174</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="E39" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>177</v>
       </c>
       <c r="G39" s="5" t="s">
         <v>22</v>
@@ -3995,10 +3986,10 @@
         <v>23</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="J39" s="8" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="K39" s="6" t="s">
         <v>17</v>
@@ -4021,22 +4012,22 @@
     </row>
     <row r="40" spans="1:16" ht="30" customHeight="1">
       <c r="A40" s="9" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B40" s="10" t="s">
         <v>17</v>
       </c>
       <c r="C40" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="D40" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="E40" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="F40" s="11" t="s">
         <v>174</v>
-      </c>
-      <c r="D40" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="E40" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="F40" s="11" t="s">
-        <v>177</v>
       </c>
       <c r="G40" s="9" t="s">
         <v>22</v>
@@ -4045,13 +4036,13 @@
         <v>23</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="J40" s="12" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="K40" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="L40" s="10" t="s">
         <v>17</v>
@@ -4071,22 +4062,22 @@
     </row>
     <row r="41" spans="1:16" ht="30" customHeight="1">
       <c r="A41" s="5" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C41" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="F41" s="7" t="s">
         <v>174</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="E41" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="F41" s="7" t="s">
-        <v>177</v>
       </c>
       <c r="G41" s="5" t="s">
         <v>16</v>
@@ -4095,13 +4086,13 @@
         <v>23</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="J41" s="8" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="K41" s="8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="L41" s="6" t="s">
         <v>17</v>
@@ -4121,22 +4112,22 @@
     </row>
     <row r="42" spans="1:16" ht="30" customHeight="1">
       <c r="A42" s="9" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B42" s="10" t="s">
         <v>17</v>
       </c>
       <c r="C42" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="D42" s="11" t="s">
+        <v>212</v>
+      </c>
+      <c r="E42" s="11" t="s">
+        <v>213</v>
+      </c>
+      <c r="F42" s="11" t="s">
         <v>174</v>
-      </c>
-      <c r="D42" s="11" t="s">
-        <v>215</v>
-      </c>
-      <c r="E42" s="11" t="s">
-        <v>216</v>
-      </c>
-      <c r="F42" s="11" t="s">
-        <v>177</v>
       </c>
       <c r="G42" s="9" t="s">
         <v>42</v>
@@ -4145,10 +4136,10 @@
         <v>23</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="J42" s="12" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="K42" s="10" t="s">
         <v>17</v>
@@ -4171,22 +4162,22 @@
     </row>
     <row r="43" spans="1:16" ht="30" customHeight="1">
       <c r="A43" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="E43" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="B43" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C43" s="7" t="s">
+      <c r="F43" s="7" t="s">
         <v>218</v>
-      </c>
-      <c r="D43" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="E43" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>221</v>
       </c>
       <c r="G43" s="5" t="s">
         <v>22</v>
@@ -4195,13 +4186,13 @@
         <v>23</v>
       </c>
       <c r="I43" s="7" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="J43" s="8" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="K43" s="8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="L43" s="6" t="s">
         <v>17</v>
@@ -4221,22 +4212,22 @@
     </row>
     <row r="44" spans="1:16" ht="30" customHeight="1">
       <c r="A44" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="B44" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C44" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="D44" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="E44" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="B44" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C44" s="11" t="s">
+      <c r="F44" s="11" t="s">
         <v>226</v>
-      </c>
-      <c r="D44" s="11" t="s">
-        <v>227</v>
-      </c>
-      <c r="E44" s="11" t="s">
-        <v>228</v>
-      </c>
-      <c r="F44" s="11" t="s">
-        <v>229</v>
       </c>
       <c r="G44" s="9" t="s">
         <v>50</v>
@@ -4245,13 +4236,13 @@
         <v>23</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="J44" s="12" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="K44" s="12" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="L44" s="10" t="s">
         <v>17</v>
@@ -4271,22 +4262,22 @@
     </row>
     <row r="45" spans="1:16" ht="30" customHeight="1">
       <c r="A45" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="F45" s="7" t="s">
         <v>233</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C45" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="D45" s="7" t="s">
-        <v>235</v>
-      </c>
-      <c r="E45" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="F45" s="7" t="s">
-        <v>236</v>
       </c>
       <c r="G45" s="5" t="s">
         <v>22</v>
@@ -4295,10 +4286,10 @@
         <v>23</v>
       </c>
       <c r="I45" s="7" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="J45" s="8" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="K45" s="6" t="s">
         <v>17</v>
@@ -4321,22 +4312,22 @@
     </row>
     <row r="46" spans="1:16" ht="30" customHeight="1">
       <c r="A46" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="B46" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C46" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="D46" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="E46" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="F46" s="11" t="s">
         <v>239</v>
-      </c>
-      <c r="B46" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C46" s="11" t="s">
-        <v>240</v>
-      </c>
-      <c r="D46" s="11" t="s">
-        <v>241</v>
-      </c>
-      <c r="E46" s="11" t="s">
-        <v>240</v>
-      </c>
-      <c r="F46" s="11" t="s">
-        <v>242</v>
       </c>
       <c r="G46" s="9" t="s">
         <v>16</v>
@@ -4345,10 +4336,10 @@
         <v>23</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="J46" s="12" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="K46" s="10" t="s">
         <v>17</v>
@@ -4366,27 +4357,27 @@
         <v>11</v>
       </c>
       <c r="P46" s="12" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="47" spans="1:16" ht="45" customHeight="1">
       <c r="A47" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="E47" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="B47" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C47" s="7" t="s">
+      <c r="F47" s="7" t="s">
         <v>247</v>
-      </c>
-      <c r="D47" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="E47" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="F47" s="7" t="s">
-        <v>250</v>
       </c>
       <c r="G47" s="5" t="s">
         <v>16</v>
@@ -4395,10 +4386,10 @@
         <v>23</v>
       </c>
       <c r="I47" s="7" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="J47" s="8" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="K47" s="6" t="s">
         <v>17</v>
@@ -4421,22 +4412,22 @@
     </row>
     <row r="48" spans="1:16" ht="30" customHeight="1">
       <c r="A48" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="B48" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C48" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="D48" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="E48" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="F48" s="11" t="s">
         <v>253</v>
-      </c>
-      <c r="B48" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C48" s="11" t="s">
-        <v>254</v>
-      </c>
-      <c r="D48" s="11" t="s">
-        <v>255</v>
-      </c>
-      <c r="E48" s="11" t="s">
-        <v>254</v>
-      </c>
-      <c r="F48" s="11" t="s">
-        <v>256</v>
       </c>
       <c r="G48" s="9" t="s">
         <v>16</v>
@@ -4445,10 +4436,10 @@
         <v>23</v>
       </c>
       <c r="I48" s="11" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="J48" s="12" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="K48" s="10" t="s">
         <v>17</v>
@@ -4471,22 +4462,22 @@
     </row>
     <row r="49" spans="1:16" ht="30" customHeight="1">
       <c r="A49" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="F49" s="7" t="s">
         <v>259</v>
-      </c>
-      <c r="B49" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C49" s="7" t="s">
-        <v>260</v>
-      </c>
-      <c r="D49" s="7" t="s">
-        <v>261</v>
-      </c>
-      <c r="E49" s="7" t="s">
-        <v>260</v>
-      </c>
-      <c r="F49" s="7" t="s">
-        <v>262</v>
       </c>
       <c r="G49" s="5" t="s">
         <v>16</v>
@@ -4495,10 +4486,10 @@
         <v>23</v>
       </c>
       <c r="I49" s="7" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="J49" s="8" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="K49" s="6" t="s">
         <v>17</v>
@@ -4521,22 +4512,22 @@
     </row>
     <row r="50" spans="1:16" ht="30" customHeight="1">
       <c r="A50" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="B50" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C50" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="D50" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="E50" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="F50" s="11" t="s">
         <v>265</v>
-      </c>
-      <c r="B50" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C50" s="11" t="s">
-        <v>266</v>
-      </c>
-      <c r="D50" s="11" t="s">
-        <v>267</v>
-      </c>
-      <c r="E50" s="11" t="s">
-        <v>266</v>
-      </c>
-      <c r="F50" s="11" t="s">
-        <v>268</v>
       </c>
       <c r="G50" s="9" t="s">
         <v>16</v>
@@ -4545,10 +4536,10 @@
         <v>23</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="J50" s="12" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="K50" s="10" t="s">
         <v>17</v>
@@ -4571,22 +4562,22 @@
     </row>
     <row r="51" spans="1:16" ht="30" customHeight="1">
       <c r="A51" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="F51" s="7" t="s">
         <v>271</v>
-      </c>
-      <c r="B51" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C51" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="D51" s="7" t="s">
-        <v>273</v>
-      </c>
-      <c r="E51" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="F51" s="7" t="s">
-        <v>274</v>
       </c>
       <c r="G51" s="5" t="s">
         <v>16</v>
@@ -4595,10 +4586,10 @@
         <v>23</v>
       </c>
       <c r="I51" s="7" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="J51" s="8" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="K51" s="6" t="s">
         <v>17</v>
@@ -4621,22 +4612,22 @@
     </row>
     <row r="52" spans="1:16" ht="30" customHeight="1">
       <c r="A52" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="B52" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C52" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="D52" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="E52" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="F52" s="11" t="s">
         <v>277</v>
-      </c>
-      <c r="B52" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C52" s="11" t="s">
-        <v>278</v>
-      </c>
-      <c r="D52" s="11" t="s">
-        <v>279</v>
-      </c>
-      <c r="E52" s="11" t="s">
-        <v>278</v>
-      </c>
-      <c r="F52" s="11" t="s">
-        <v>280</v>
       </c>
       <c r="G52" s="9" t="s">
         <v>16</v>
@@ -4645,10 +4636,10 @@
         <v>23</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="J52" s="12" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="K52" s="10" t="s">
         <v>17</v>
@@ -4671,22 +4662,22 @@
     </row>
     <row r="53" spans="1:16" ht="30" customHeight="1">
       <c r="A53" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="F53" s="7" t="s">
         <v>283</v>
-      </c>
-      <c r="B53" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C53" s="7" t="s">
-        <v>284</v>
-      </c>
-      <c r="D53" s="7" t="s">
-        <v>285</v>
-      </c>
-      <c r="E53" s="7" t="s">
-        <v>284</v>
-      </c>
-      <c r="F53" s="7" t="s">
-        <v>286</v>
       </c>
       <c r="G53" s="5" t="s">
         <v>16</v>
@@ -4695,10 +4686,10 @@
         <v>23</v>
       </c>
       <c r="I53" s="7" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="J53" s="8" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="K53" s="6" t="s">
         <v>17</v>
@@ -4721,22 +4712,22 @@
     </row>
     <row r="54" spans="1:16" ht="30" customHeight="1">
       <c r="A54" s="9" t="s">
+        <v>286</v>
+      </c>
+      <c r="B54" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C54" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="D54" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="E54" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="F54" s="11" t="s">
         <v>289</v>
-      </c>
-      <c r="B54" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C54" s="11" t="s">
-        <v>290</v>
-      </c>
-      <c r="D54" s="11" t="s">
-        <v>291</v>
-      </c>
-      <c r="E54" s="11" t="s">
-        <v>290</v>
-      </c>
-      <c r="F54" s="11" t="s">
-        <v>292</v>
       </c>
       <c r="G54" s="9" t="s">
         <v>16</v>
@@ -4745,10 +4736,10 @@
         <v>23</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="J54" s="12" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="K54" s="10" t="s">
         <v>17</v>
@@ -4771,22 +4762,22 @@
     </row>
     <row r="55" spans="1:16" ht="30" customHeight="1">
       <c r="A55" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="E55" s="7" t="s">
         <v>295</v>
       </c>
-      <c r="B55" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C55" s="7" t="s">
+      <c r="F55" s="7" t="s">
         <v>296</v>
-      </c>
-      <c r="D55" s="7" t="s">
-        <v>297</v>
-      </c>
-      <c r="E55" s="7" t="s">
-        <v>298</v>
-      </c>
-      <c r="F55" s="7" t="s">
-        <v>299</v>
       </c>
       <c r="G55" s="5" t="s">
         <v>16</v>
@@ -4795,10 +4786,10 @@
         <v>23</v>
       </c>
       <c r="I55" s="7" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="J55" s="8" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="K55" s="6" t="s">
         <v>17</v>
@@ -4821,22 +4812,22 @@
     </row>
     <row r="56" spans="1:16" ht="30" customHeight="1">
       <c r="A56" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="B56" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C56" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="D56" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="E56" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="F56" s="11" t="s">
         <v>302</v>
-      </c>
-      <c r="B56" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C56" s="11" t="s">
-        <v>303</v>
-      </c>
-      <c r="D56" s="11" t="s">
-        <v>304</v>
-      </c>
-      <c r="E56" s="11" t="s">
-        <v>303</v>
-      </c>
-      <c r="F56" s="11" t="s">
-        <v>305</v>
       </c>
       <c r="G56" s="9" t="s">
         <v>16</v>
@@ -4845,10 +4836,10 @@
         <v>23</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="J56" s="12" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K56" s="10" t="s">
         <v>17</v>
@@ -4871,22 +4862,22 @@
     </row>
     <row r="57" spans="1:16" ht="30" customHeight="1">
       <c r="A57" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="E57" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="F57" s="7" t="s">
         <v>308</v>
-      </c>
-      <c r="B57" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C57" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>310</v>
-      </c>
-      <c r="E57" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="F57" s="7" t="s">
-        <v>311</v>
       </c>
       <c r="G57" s="5" t="s">
         <v>16</v>
@@ -4895,10 +4886,10 @@
         <v>23</v>
       </c>
       <c r="I57" s="7" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="J57" s="8" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="K57" s="6" t="s">
         <v>17</v>
@@ -4937,7 +4928,7 @@
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
     <col min="2" max="2" width="21.7109375" customWidth="1"/>
     <col min="3" max="3" width="23.7109375" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="4" max="4" width="27.7109375" customWidth="1"/>
     <col min="5" max="5" width="28.7109375" customWidth="1"/>
     <col min="6" max="6" width="42.7109375" customWidth="1"/>
     <col min="7" max="7" width="26.7109375" customWidth="1"/>
@@ -4951,7 +4942,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="32" customHeight="1">
       <c r="C1" s="1" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -4969,13 +4960,13 @@
     </row>
     <row r="2" spans="1:16">
       <c r="C2" s="2" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="F2" s="3">
         <v>55</v>
@@ -4983,41 +4974,41 @@
     </row>
     <row r="3" spans="1:16">
       <c r="C3" s="2" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="4" spans="1:16">
       <c r="C4" s="2" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="5" spans="1:16">
       <c r="C5" s="2" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="F5" s="3">
         <v>1</v>
@@ -5025,13 +5016,13 @@
     </row>
     <row r="6" spans="1:16">
       <c r="C6" s="2" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="F6" s="3">
         <v>128</v>
@@ -5095,28 +5086,28 @@
         <v>17</v>
       </c>
       <c r="C9" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="F9" s="7" t="s">
         <v>332</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>333</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>334</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>335</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>16</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="K9" s="6" t="s">
         <v>17</v>
@@ -5145,31 +5136,31 @@
         <v>17</v>
       </c>
       <c r="C10" s="11" t="s">
+        <v>336</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>337</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>338</v>
+      </c>
+      <c r="F10" s="11" t="s">
         <v>339</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>340</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>341</v>
-      </c>
-      <c r="F10" s="11" t="s">
-        <v>342</v>
       </c>
       <c r="G10" s="9" t="s">
         <v>22</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="L10" s="10" t="s">
         <v>17</v>
@@ -5195,25 +5186,25 @@
         <v>17</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>22</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>17</v>
@@ -5245,28 +5236,28 @@
         <v>17</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="G12" s="9" t="s">
         <v>22</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J12" s="12" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="K12" s="10" t="s">
         <v>17</v>
@@ -5295,25 +5286,25 @@
         <v>17</v>
       </c>
       <c r="C13" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="F13" s="7" t="s">
         <v>174</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>353</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>177</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>16</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>17</v>
@@ -5345,31 +5336,31 @@
         <v>17</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="G14" s="9" t="s">
         <v>22</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="K14" s="12" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="L14" s="10" t="s">
         <v>17</v>
@@ -5414,7 +5405,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="32" customHeight="1">
       <c r="D1" s="1" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -5423,13 +5414,13 @@
     </row>
     <row r="2" spans="1:8">
       <c r="D2" s="2" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="H2" s="13">
         <v>1</v>
@@ -5437,13 +5428,13 @@
     </row>
     <row r="3" spans="1:8">
       <c r="D3" s="2" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="H3" s="15">
         <f>TotalCost/BoardQty</f>
@@ -5452,13 +5443,13 @@
     </row>
     <row r="4" spans="1:8">
       <c r="D4" s="2" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="H4" s="16">
         <f>SUM(H10:H58)</f>
@@ -5467,23 +5458,23 @@
     </row>
     <row r="5" spans="1:8">
       <c r="D5" s="2" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="D6" s="2" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="17" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -5507,16 +5498,16 @@
         <v>5</v>
       </c>
       <c r="E9" s="18" t="s">
+        <v>358</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>360</v>
+      </c>
+      <c r="H9" s="18" t="s">
         <v>361</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>362</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>363</v>
-      </c>
-      <c r="H9" s="18" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -5725,7 +5716,7 @@
         <v>79</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="D19" s="19" t="s">
         <v>80</v>
@@ -5741,13 +5732,13 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="B20" s="19" t="s">
-        <v>86</v>
-      </c>
       <c r="C20" s="19" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="D20" s="19" t="s">
         <v>80</v>
@@ -5763,16 +5754,16 @@
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1">
       <c r="A21" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="D21" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="D21" s="19" t="s">
+      <c r="E21" s="19" t="s">
         <v>92</v>
-      </c>
-      <c r="E21" s="19" t="s">
-        <v>93</v>
       </c>
       <c r="F21" s="19">
         <f>BoardQty*1</f>
@@ -5785,16 +5776,16 @@
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1">
       <c r="A22" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="B22" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="D22" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="D22" s="19" t="s">
+      <c r="E22" s="19" t="s">
         <v>99</v>
-      </c>
-      <c r="E22" s="19" t="s">
-        <v>100</v>
       </c>
       <c r="F22" s="19">
         <f>BoardQty*1</f>
@@ -5807,16 +5798,16 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="D23" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="D23" s="19" t="s">
+      <c r="E23" s="19" t="s">
         <v>106</v>
-      </c>
-      <c r="E23" s="19" t="s">
-        <v>107</v>
       </c>
       <c r="F23" s="19">
         <f>BoardQty*1</f>
@@ -5829,16 +5820,16 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="B24" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="D24" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="D24" s="19" t="s">
-        <v>113</v>
-      </c>
       <c r="E24" s="19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F24" s="19">
         <f>BoardQty*1</f>
@@ -5851,16 +5842,16 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="B25" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="D25" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="D25" s="19" t="s">
+      <c r="E25" s="19" t="s">
         <v>119</v>
-      </c>
-      <c r="E25" s="19" t="s">
-        <v>120</v>
       </c>
       <c r="F25" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -5873,16 +5864,16 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="B26" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="B26" s="19" t="s">
+      <c r="D26" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="D26" s="19" t="s">
+      <c r="E26" s="19" t="s">
         <v>126</v>
-      </c>
-      <c r="E26" s="19" t="s">
-        <v>127</v>
       </c>
       <c r="F26" s="19">
         <f>CEILING(BoardQty*6,1)</f>
@@ -5895,13 +5886,13 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="19" t="s">
+        <v>131</v>
+      </c>
+      <c r="B27" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="B27" s="19" t="s">
+      <c r="D27" s="19" t="s">
         <v>133</v>
-      </c>
-      <c r="D27" s="19" t="s">
-        <v>134</v>
       </c>
       <c r="F27" s="19">
         <f>BoardQty*1</f>
@@ -5914,16 +5905,16 @@
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1">
       <c r="A28" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="D28" s="19" t="s">
         <v>137</v>
       </c>
-      <c r="B28" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="D28" s="19" t="s">
+      <c r="E28" s="19" t="s">
         <v>138</v>
-      </c>
-      <c r="E28" s="19" t="s">
-        <v>139</v>
       </c>
       <c r="F28" s="19">
         <f>BoardQty*1</f>
@@ -5936,19 +5927,19 @@
     </row>
     <row r="29" spans="1:8" ht="30" customHeight="1">
       <c r="A29" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="C29" s="19" t="s">
+        <v>363</v>
+      </c>
+      <c r="D29" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="B29" s="19" t="s">
-        <v>142</v>
-      </c>
-      <c r="C29" s="19" t="s">
-        <v>366</v>
-      </c>
-      <c r="D29" s="19" t="s">
+      <c r="E29" s="19" t="s">
         <v>144</v>
-      </c>
-      <c r="E29" s="19" t="s">
-        <v>145</v>
       </c>
       <c r="F29" s="19">
         <f>BoardQty*1</f>
@@ -5961,19 +5952,19 @@
     </row>
     <row r="30" spans="1:8" ht="30" customHeight="1">
       <c r="A30" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="B30" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="C30" s="19" t="s">
+        <v>364</v>
+      </c>
+      <c r="D30" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="E30" s="19" t="s">
         <v>149</v>
-      </c>
-      <c r="B30" s="19" t="s">
-        <v>148</v>
-      </c>
-      <c r="C30" s="19" t="s">
-        <v>367</v>
-      </c>
-      <c r="D30" s="19" t="s">
-        <v>150</v>
-      </c>
-      <c r="E30" s="19" t="s">
-        <v>151</v>
       </c>
       <c r="F30" s="19">
         <f>BoardQty*1</f>
@@ -5986,16 +5977,16 @@
     </row>
     <row r="31" spans="1:8" ht="30" customHeight="1">
       <c r="A31" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="B31" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="D31" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="E31" s="19" t="s">
         <v>154</v>
-      </c>
-      <c r="B31" s="19" t="s">
-        <v>155</v>
-      </c>
-      <c r="D31" s="19" t="s">
-        <v>156</v>
-      </c>
-      <c r="E31" s="19" t="s">
-        <v>157</v>
       </c>
       <c r="F31" s="19">
         <f>CEILING(BoardQty*4,1)</f>
@@ -6008,16 +5999,16 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="B32" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="D32" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="E32" s="19" t="s">
         <v>161</v>
-      </c>
-      <c r="B32" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="D32" s="19" t="s">
-        <v>163</v>
-      </c>
-      <c r="E32" s="19" t="s">
-        <v>164</v>
       </c>
       <c r="F32" s="19">
         <f>BoardQty*1</f>
@@ -6030,16 +6021,16 @@
     </row>
     <row r="33" spans="1:8">
       <c r="A33" s="19" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B33" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D33" s="19" t="s">
+        <v>167</v>
+      </c>
+      <c r="E33" s="19" t="s">
         <v>168</v>
-      </c>
-      <c r="D33" s="19" t="s">
-        <v>170</v>
-      </c>
-      <c r="E33" s="19" t="s">
-        <v>171</v>
       </c>
       <c r="F33" s="19">
         <f>BoardQty*1</f>
@@ -6052,16 +6043,16 @@
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="19" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F34" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -6074,16 +6065,16 @@
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="19" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F35" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -6096,16 +6087,16 @@
     </row>
     <row r="36" spans="1:8">
       <c r="A36" s="19" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F36" s="19">
         <f>BoardQty*1</f>
@@ -6118,16 +6109,16 @@
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="19" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F37" s="19">
         <f>CEILING(BoardQty*3,1)</f>
@@ -6140,16 +6131,16 @@
     </row>
     <row r="38" spans="1:8">
       <c r="A38" s="19" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F38" s="19">
         <f>CEILING(BoardQty*5,1)</f>
@@ -6162,16 +6153,16 @@
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="19" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F39" s="19">
         <f>CEILING(BoardQty*5,1)</f>
@@ -6184,16 +6175,16 @@
     </row>
     <row r="40" spans="1:8">
       <c r="A40" s="19" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F40" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -6206,16 +6197,16 @@
     </row>
     <row r="41" spans="1:8">
       <c r="A41" s="19" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C41" s="19" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D41" s="19" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F41" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -6228,16 +6219,16 @@
     </row>
     <row r="42" spans="1:8">
       <c r="A42" s="19" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D42" s="19" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F42" s="19">
         <f>BoardQty*1</f>
@@ -6250,16 +6241,16 @@
     </row>
     <row r="43" spans="1:8">
       <c r="A43" s="19" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C43" s="19" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D43" s="19" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F43" s="19">
         <f>CEILING(BoardQty*5,1)</f>
@@ -6272,16 +6263,16 @@
     </row>
     <row r="44" spans="1:8" ht="30" customHeight="1">
       <c r="A44" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="B44" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="D44" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="E44" s="19" t="s">
         <v>219</v>
-      </c>
-      <c r="B44" s="19" t="s">
-        <v>220</v>
-      </c>
-      <c r="D44" s="19" t="s">
-        <v>221</v>
-      </c>
-      <c r="E44" s="19" t="s">
-        <v>222</v>
       </c>
       <c r="F44" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -6294,16 +6285,16 @@
     </row>
     <row r="45" spans="1:8" ht="30" customHeight="1">
       <c r="A45" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="B45" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="D45" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="E45" s="19" t="s">
         <v>227</v>
-      </c>
-      <c r="B45" s="19" t="s">
-        <v>228</v>
-      </c>
-      <c r="D45" s="19" t="s">
-        <v>229</v>
-      </c>
-      <c r="E45" s="19" t="s">
-        <v>230</v>
       </c>
       <c r="F45" s="19">
         <f>CEILING(BoardQty*6,1)</f>
@@ -6316,16 +6307,16 @@
     </row>
     <row r="46" spans="1:8">
       <c r="A46" s="19" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B46" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="D46" s="19" t="s">
+        <v>233</v>
+      </c>
+      <c r="E46" s="19" t="s">
         <v>234</v>
-      </c>
-      <c r="D46" s="19" t="s">
-        <v>236</v>
-      </c>
-      <c r="E46" s="19" t="s">
-        <v>237</v>
       </c>
       <c r="F46" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -6338,16 +6329,16 @@
     </row>
     <row r="47" spans="1:8">
       <c r="A47" s="19" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B47" s="19" t="s">
+        <v>237</v>
+      </c>
+      <c r="D47" s="19" t="s">
+        <v>239</v>
+      </c>
+      <c r="E47" s="19" t="s">
         <v>240</v>
-      </c>
-      <c r="D47" s="19" t="s">
-        <v>242</v>
-      </c>
-      <c r="E47" s="19" t="s">
-        <v>243</v>
       </c>
       <c r="F47" s="19">
         <f>BoardQty*1</f>
@@ -6360,16 +6351,16 @@
     </row>
     <row r="48" spans="1:8" ht="45" customHeight="1">
       <c r="A48" s="19" t="s">
+        <v>245</v>
+      </c>
+      <c r="B48" s="19" t="s">
+        <v>246</v>
+      </c>
+      <c r="D48" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="E48" s="19" t="s">
         <v>248</v>
-      </c>
-      <c r="B48" s="19" t="s">
-        <v>249</v>
-      </c>
-      <c r="D48" s="19" t="s">
-        <v>250</v>
-      </c>
-      <c r="E48" s="19" t="s">
-        <v>251</v>
       </c>
       <c r="F48" s="19">
         <f>BoardQty*1</f>
@@ -6382,19 +6373,19 @@
     </row>
     <row r="49" spans="1:8" ht="30" customHeight="1">
       <c r="A49" s="19" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B49" s="19" t="s">
+        <v>251</v>
+      </c>
+      <c r="C49" s="19" t="s">
+        <v>366</v>
+      </c>
+      <c r="D49" s="19" t="s">
+        <v>253</v>
+      </c>
+      <c r="E49" s="19" t="s">
         <v>254</v>
-      </c>
-      <c r="C49" s="19" t="s">
-        <v>369</v>
-      </c>
-      <c r="D49" s="19" t="s">
-        <v>256</v>
-      </c>
-      <c r="E49" s="19" t="s">
-        <v>257</v>
       </c>
       <c r="F49" s="19">
         <f>BoardQty*1</f>
@@ -6407,19 +6398,19 @@
     </row>
     <row r="50" spans="1:8" ht="30" customHeight="1">
       <c r="A50" s="19" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="B50" s="19" t="s">
+        <v>257</v>
+      </c>
+      <c r="C50" s="19" t="s">
+        <v>367</v>
+      </c>
+      <c r="D50" s="19" t="s">
+        <v>259</v>
+      </c>
+      <c r="E50" s="19" t="s">
         <v>260</v>
-      </c>
-      <c r="C50" s="19" t="s">
-        <v>370</v>
-      </c>
-      <c r="D50" s="19" t="s">
-        <v>262</v>
-      </c>
-      <c r="E50" s="19" t="s">
-        <v>263</v>
       </c>
       <c r="F50" s="19">
         <f>BoardQty*1</f>
@@ -6432,16 +6423,16 @@
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="19" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B51" s="19" t="s">
+        <v>263</v>
+      </c>
+      <c r="D51" s="19" t="s">
+        <v>265</v>
+      </c>
+      <c r="E51" s="19" t="s">
         <v>266</v>
-      </c>
-      <c r="D51" s="19" t="s">
-        <v>268</v>
-      </c>
-      <c r="E51" s="19" t="s">
-        <v>269</v>
       </c>
       <c r="F51" s="19">
         <f>BoardQty*1</f>
@@ -6454,16 +6445,16 @@
     </row>
     <row r="52" spans="1:8" ht="30" customHeight="1">
       <c r="A52" s="19" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="B52" s="19" t="s">
+        <v>269</v>
+      </c>
+      <c r="D52" s="19" t="s">
+        <v>271</v>
+      </c>
+      <c r="E52" s="19" t="s">
         <v>272</v>
-      </c>
-      <c r="D52" s="19" t="s">
-        <v>274</v>
-      </c>
-      <c r="E52" s="19" t="s">
-        <v>275</v>
       </c>
       <c r="F52" s="19">
         <f>BoardQty*1</f>
@@ -6476,19 +6467,19 @@
     </row>
     <row r="53" spans="1:8" ht="30" customHeight="1">
       <c r="A53" s="19" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="B53" s="19" t="s">
+        <v>275</v>
+      </c>
+      <c r="C53" s="19" t="s">
+        <v>368</v>
+      </c>
+      <c r="D53" s="19" t="s">
+        <v>277</v>
+      </c>
+      <c r="E53" s="19" t="s">
         <v>278</v>
-      </c>
-      <c r="C53" s="19" t="s">
-        <v>371</v>
-      </c>
-      <c r="D53" s="19" t="s">
-        <v>280</v>
-      </c>
-      <c r="E53" s="19" t="s">
-        <v>281</v>
       </c>
       <c r="F53" s="19">
         <f>BoardQty*1</f>
@@ -6501,19 +6492,19 @@
     </row>
     <row r="54" spans="1:8" ht="30" customHeight="1">
       <c r="A54" s="19" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="B54" s="19" t="s">
+        <v>281</v>
+      </c>
+      <c r="C54" s="19" t="s">
+        <v>369</v>
+      </c>
+      <c r="D54" s="19" t="s">
+        <v>283</v>
+      </c>
+      <c r="E54" s="19" t="s">
         <v>284</v>
-      </c>
-      <c r="C54" s="19" t="s">
-        <v>372</v>
-      </c>
-      <c r="D54" s="19" t="s">
-        <v>286</v>
-      </c>
-      <c r="E54" s="19" t="s">
-        <v>287</v>
       </c>
       <c r="F54" s="19">
         <f>BoardQty*1</f>
@@ -6526,19 +6517,19 @@
     </row>
     <row r="55" spans="1:8" ht="30" customHeight="1">
       <c r="A55" s="19" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="B55" s="19" t="s">
+        <v>287</v>
+      </c>
+      <c r="C55" s="19" t="s">
+        <v>370</v>
+      </c>
+      <c r="D55" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="E55" s="19" t="s">
         <v>290</v>
-      </c>
-      <c r="C55" s="19" t="s">
-        <v>373</v>
-      </c>
-      <c r="D55" s="19" t="s">
-        <v>292</v>
-      </c>
-      <c r="E55" s="19" t="s">
-        <v>293</v>
       </c>
       <c r="F55" s="19">
         <f>BoardQty*1</f>
@@ -6551,16 +6542,16 @@
     </row>
     <row r="56" spans="1:8" ht="30" customHeight="1">
       <c r="A56" s="19" t="s">
+        <v>294</v>
+      </c>
+      <c r="B56" s="19" t="s">
+        <v>295</v>
+      </c>
+      <c r="D56" s="19" t="s">
+        <v>296</v>
+      </c>
+      <c r="E56" s="19" t="s">
         <v>297</v>
-      </c>
-      <c r="B56" s="19" t="s">
-        <v>298</v>
-      </c>
-      <c r="D56" s="19" t="s">
-        <v>299</v>
-      </c>
-      <c r="E56" s="19" t="s">
-        <v>300</v>
       </c>
       <c r="F56" s="19">
         <f>BoardQty*1</f>
@@ -6573,16 +6564,16 @@
     </row>
     <row r="57" spans="1:8">
       <c r="A57" s="19" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B57" s="19" t="s">
+        <v>300</v>
+      </c>
+      <c r="D57" s="19" t="s">
+        <v>302</v>
+      </c>
+      <c r="E57" s="19" t="s">
         <v>303</v>
-      </c>
-      <c r="D57" s="19" t="s">
-        <v>305</v>
-      </c>
-      <c r="E57" s="19" t="s">
-        <v>306</v>
       </c>
       <c r="F57" s="19">
         <f>BoardQty*1</f>
@@ -6595,19 +6586,19 @@
     </row>
     <row r="58" spans="1:8" ht="30" customHeight="1">
       <c r="A58" s="19" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="B58" s="19" t="s">
+        <v>306</v>
+      </c>
+      <c r="C58" s="19" t="s">
+        <v>371</v>
+      </c>
+      <c r="D58" s="19" t="s">
+        <v>308</v>
+      </c>
+      <c r="E58" s="19" t="s">
         <v>309</v>
-      </c>
-      <c r="C58" s="19" t="s">
-        <v>374</v>
-      </c>
-      <c r="D58" s="19" t="s">
-        <v>311</v>
-      </c>
-      <c r="E58" s="19" t="s">
-        <v>312</v>
       </c>
       <c r="F58" s="19">
         <f>BoardQty*1</f>
@@ -6620,15 +6611,15 @@
     </row>
     <row r="61" spans="1:8">
       <c r="A61" s="21" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="B61" s="22" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
     </row>
     <row r="62" spans="1:8">
       <c r="A62" s="23" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
     </row>
   </sheetData>
@@ -6942,7 +6933,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="32" customHeight="1">
       <c r="D1" s="1" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -6951,13 +6942,13 @@
     </row>
     <row r="2" spans="1:8">
       <c r="D2" s="2" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="H2" s="13">
         <v>1</v>
@@ -6965,13 +6956,13 @@
     </row>
     <row r="3" spans="1:8">
       <c r="D3" s="2" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="H3" s="15">
         <f>TotalCost/BoardQty</f>
@@ -6980,13 +6971,13 @@
     </row>
     <row r="4" spans="1:8">
       <c r="D4" s="2" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="H4" s="16">
         <f>SUM(H10:H15)</f>
@@ -6995,23 +6986,23 @@
     </row>
     <row r="5" spans="1:8">
       <c r="D5" s="2" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="D6" s="2" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="17" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -7035,30 +7026,30 @@
         <v>5</v>
       </c>
       <c r="E9" s="18" t="s">
+        <v>358</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>360</v>
+      </c>
+      <c r="H9" s="18" t="s">
         <v>361</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>362</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>363</v>
-      </c>
-      <c r="H9" s="18" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1">
       <c r="A10" s="19" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="B10" s="19" t="s">
+        <v>331</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>332</v>
+      </c>
+      <c r="E10" s="19" t="s">
         <v>334</v>
-      </c>
-      <c r="D10" s="19" t="s">
-        <v>335</v>
-      </c>
-      <c r="E10" s="19" t="s">
-        <v>337</v>
       </c>
       <c r="F10" s="19">
         <f>BoardQty*1</f>
@@ -7071,19 +7062,19 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="19" t="s">
+        <v>337</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>338</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>378</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>339</v>
+      </c>
+      <c r="E11" s="19" t="s">
         <v>340</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>341</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>381</v>
-      </c>
-      <c r="D11" s="19" t="s">
-        <v>342</v>
-      </c>
-      <c r="E11" s="19" t="s">
-        <v>343</v>
       </c>
       <c r="F11" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -7096,13 +7087,13 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="19" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F12" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -7115,16 +7106,16 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="19" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F13" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -7137,16 +7128,16 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="19" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F14" s="19">
         <f>BoardQty*1</f>
@@ -7159,16 +7150,16 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="19" t="s">
+        <v>351</v>
+      </c>
+      <c r="B15" s="19" t="s">
+        <v>352</v>
+      </c>
+      <c r="D15" s="19" t="s">
+        <v>353</v>
+      </c>
+      <c r="E15" s="19" t="s">
         <v>354</v>
-      </c>
-      <c r="B15" s="19" t="s">
-        <v>355</v>
-      </c>
-      <c r="D15" s="19" t="s">
-        <v>356</v>
-      </c>
-      <c r="E15" s="19" t="s">
-        <v>357</v>
       </c>
       <c r="F15" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -7181,15 +7172,15 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="21" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="23" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
     </row>
   </sheetData>
@@ -7249,77 +7240,77 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="7" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="5" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="8" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="6" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="24" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="25" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="26" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="27" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="28" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="29" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="30" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="31" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="32" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ pedalboard/pedalboard-hw@3850a8c2391c59a8afc3a21d9ad2627a5685ea24 🚀
</commit_message>
<xml_diff>
--- a/latest/BoM/Costs/pedalboard-hw-bom.xlsx
+++ b/latest/BoM/Costs/pedalboard-hw-bom.xlsx
@@ -1420,10 +1420,10 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2026-05-12 07:06:18</t>
-  </si>
-  <si>
-    <t>KiCost® v1.1.20 + KiBot v1.8.6</t>
+    <t>2026-05-13 11:26:00</t>
+  </si>
+  <si>
+    <t>KiCost® v1.1.20 + KiBot v1.9.0</t>
   </si>
   <si>
     <t>5-pin DIN connector (5-pin DIN-5 stereo)</t>

</xml_diff>